<commit_message>
finition de la première phase
</commit_message>
<xml_diff>
--- a/Project.xlsx
+++ b/Project.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ac5112b48b0b9b87/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="11_01AABC5FF85B2F9B595C382F1D8B29F5AE293287" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8FC0A6C-2814-42A8-B247-AA9AC6EF67B8}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="11_01AABC5FF85B2F9B595C382F1D8B29F5AE293287" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2344A57D-9B07-4FB6-A3C7-B0C5C564E492}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="project_parameters" sheetId="1" r:id="rId1"/>
@@ -166,10 +166,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="_-* #,##0\ [$€-40C]_-;\-* #,##0\ [$€-40C]_-;_-* &quot;-&quot;??\ [$€-40C]_-;_-@_-"/>
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -188,6 +189,13 @@
     <font>
       <b/>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -217,18 +225,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Milliers" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -533,14 +542,14 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
-    <col min="2" max="2" width="26.28515625" customWidth="1"/>
+    <col min="2" max="2" width="28.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:7" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
@@ -556,8 +565,8 @@
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1">
-        <v>7622450.8618705189</v>
+      <c r="B3" s="4">
+        <v>5000000000</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -589,6 +598,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -602,17 +612,17 @@
     <col min="4" max="4" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>12</v>
       </c>
     </row>
@@ -802,46 +812,46 @@
     <col min="7" max="7" width="22.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4">
+    <row r="2" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="5">
-        <v>533571.56033093634</v>
-      </c>
-      <c r="E2" s="4">
+      <c r="D2" s="4">
+        <v>350000000</v>
+      </c>
+      <c r="E2" s="3">
         <v>0.95</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="3">
         <v>12</v>
       </c>
     </row>
@@ -855,8 +865,8 @@
       <c r="C3" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="1">
-        <v>762245.08618705196</v>
+      <c r="D3" s="4">
+        <v>500000000</v>
       </c>
       <c r="E3">
         <v>0.98</v>
@@ -868,23 +878,23 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4">
+    <row r="4" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="5">
-        <v>457347.05171223113</v>
-      </c>
-      <c r="E4" s="4">
+      <c r="D4" s="4">
+        <v>300000000</v>
+      </c>
+      <c r="E4" s="3">
         <v>0.9</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="3">
         <v>8</v>
       </c>
     </row>
@@ -898,8 +908,8 @@
       <c r="C5" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="1">
-        <v>381122.54309352598</v>
+      <c r="D5" s="4">
+        <v>250000000</v>
       </c>
       <c r="E5">
         <v>0.85</v>
@@ -921,8 +931,8 @@
       <c r="C6" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="1">
-        <v>609796.06894964154</v>
+      <c r="D6" s="4">
+        <v>400000000</v>
       </c>
       <c r="E6">
         <v>0.92</v>
@@ -944,8 +954,8 @@
       <c r="C7" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="1">
-        <v>304898.03447482077</v>
+      <c r="D7" s="4">
+        <v>200000000</v>
       </c>
       <c r="E7">
         <v>0.88</v>
@@ -967,8 +977,8 @@
       <c r="C8" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="1">
-        <v>228673.52585611556</v>
+      <c r="D8" s="4">
+        <v>150000000</v>
       </c>
       <c r="E8">
         <v>0.8</v>
@@ -990,8 +1000,8 @@
       <c r="C9" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="1">
-        <v>686020.57756834675</v>
+      <c r="D9" s="4">
+        <v>450000000</v>
       </c>
       <c r="E9">
         <v>0.97</v>
@@ -1003,23 +1013,23 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="4">
+    <row r="10" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
         <v>9</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="5">
-        <v>182938.82068489245</v>
-      </c>
-      <c r="E10" s="4">
+      <c r="D10" s="4">
+        <v>120000000</v>
+      </c>
+      <c r="E10" s="3">
         <v>0.75</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="3">
         <v>5</v>
       </c>
     </row>
@@ -1033,8 +1043,8 @@
       <c r="C11" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="1">
-        <v>640285.8723971236</v>
+      <c r="D11" s="4">
+        <v>420000000</v>
       </c>
       <c r="E11">
         <v>0.93</v>
@@ -1061,14 +1071,14 @@
     <col min="3" max="3" width="25.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1197,14 +1207,14 @@
     <col min="3" max="3" width="18.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>37</v>
       </c>
     </row>

</xml_diff>